<commit_message>
added remaining brackets and updated score for first game to validate it is working
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D805A157-9AE0-43CE-B6BC-31C4601DBDF0}"/>
+  <bookViews>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="madness" state="visible" r:id="rId4"/>
+    <sheet name="madness" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="80">
   <si>
     <t>2026 March Madness Bracket</t>
   </si>
@@ -248,19 +252,22 @@
   </si>
   <si>
     <t>Tennessee State</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -623,16 +630,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AM72"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -667,7 +674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B7">
         <v>1</v>
       </c>
@@ -681,7 +688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E8" t="s">
         <v>9</v>
       </c>
@@ -689,7 +696,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B9">
         <v>16</v>
       </c>
@@ -703,7 +710,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H10" t="s">
         <v>9</v>
       </c>
@@ -711,13 +718,16 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B11">
         <v>8</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
+      <c r="D11">
+        <v>64</v>
+      </c>
       <c r="AL11" t="s">
         <v>13</v>
       </c>
@@ -725,21 +735,24 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E12" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="AJ12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B13">
         <v>9</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>
       </c>
+      <c r="D13">
+        <v>66</v>
+      </c>
       <c r="AL13" t="s">
         <v>15</v>
       </c>
@@ -747,7 +760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K14" t="s">
         <v>9</v>
       </c>
@@ -755,7 +768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B15">
         <v>5</v>
       </c>
@@ -769,7 +782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E16" t="s">
         <v>9</v>
       </c>
@@ -777,7 +790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B17">
         <v>12</v>
       </c>
@@ -791,7 +804,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H18" t="s">
         <v>9</v>
       </c>
@@ -799,13 +812,16 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B19">
         <v>4</v>
       </c>
       <c r="C19" t="s">
         <v>20</v>
       </c>
+      <c r="P19" t="s">
+        <v>79</v>
+      </c>
       <c r="AL19" t="s">
         <v>21</v>
       </c>
@@ -813,7 +829,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E20" t="s">
         <v>9</v>
       </c>
@@ -821,7 +837,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B21">
         <v>13</v>
       </c>
@@ -835,7 +851,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K22" t="s">
         <v>24</v>
       </c>
@@ -849,7 +865,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B23">
         <v>6</v>
       </c>
@@ -863,7 +879,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" t="s">
         <v>9</v>
       </c>
@@ -871,7 +887,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B25">
         <v>11</v>
       </c>
@@ -885,7 +901,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H26" t="s">
         <v>9</v>
       </c>
@@ -893,7 +909,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B27">
         <v>3</v>
       </c>
@@ -907,7 +923,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E28" t="s">
         <v>9</v>
       </c>
@@ -915,7 +931,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B29">
         <v>14</v>
       </c>
@@ -929,7 +945,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K30" t="s">
         <v>9</v>
       </c>
@@ -937,7 +953,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B31">
         <v>7</v>
       </c>
@@ -951,7 +967,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E32" t="s">
         <v>9</v>
       </c>
@@ -959,7 +975,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B33">
         <v>10</v>
       </c>
@@ -973,7 +989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H34" t="s">
         <v>9</v>
       </c>
@@ -981,7 +997,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B35">
         <v>2</v>
       </c>
@@ -995,7 +1011,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E36" t="s">
         <v>9</v>
       </c>
@@ -1003,7 +1019,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B37">
         <v>15</v>
       </c>
@@ -1017,7 +1033,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="15:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="O39" t="s">
         <v>9</v>
       </c>
@@ -1025,7 +1041,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B42">
         <v>1</v>
       </c>
@@ -1039,7 +1055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E43" t="s">
         <v>9</v>
       </c>
@@ -1047,7 +1063,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B44">
         <v>16</v>
       </c>
@@ -1064,7 +1080,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H45" t="s">
         <v>9</v>
       </c>
@@ -1072,7 +1088,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B46">
         <v>8</v>
       </c>
@@ -1089,7 +1105,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E47" t="s">
         <v>9</v>
       </c>
@@ -1097,7 +1113,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B48">
         <v>9</v>
       </c>
@@ -1111,7 +1127,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K49" t="s">
         <v>9</v>
       </c>
@@ -1119,7 +1135,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B50">
         <v>5</v>
       </c>
@@ -1136,7 +1152,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E51" t="s">
         <v>9</v>
       </c>
@@ -1144,7 +1160,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B52">
         <v>12</v>
       </c>
@@ -1158,7 +1174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H53" t="s">
         <v>9</v>
       </c>
@@ -1166,7 +1182,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B54">
         <v>4</v>
       </c>
@@ -1183,7 +1199,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E55" t="s">
         <v>9</v>
       </c>
@@ -1191,7 +1207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B56">
         <v>13</v>
       </c>
@@ -1205,7 +1221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K57" t="s">
         <v>61</v>
       </c>
@@ -1219,7 +1235,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B58">
         <v>6</v>
       </c>
@@ -1233,7 +1249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E59" t="s">
         <v>9</v>
       </c>
@@ -1241,7 +1257,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B60">
         <v>11</v>
       </c>
@@ -1255,7 +1271,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H61" t="s">
         <v>9</v>
       </c>
@@ -1263,7 +1279,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B62">
         <v>3</v>
       </c>
@@ -1277,7 +1293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E63" t="s">
         <v>9</v>
       </c>
@@ -1285,7 +1301,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B64">
         <v>14</v>
       </c>
@@ -1299,7 +1315,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K65" t="s">
         <v>9</v>
       </c>
@@ -1307,7 +1323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B66">
         <v>7</v>
       </c>
@@ -1321,7 +1337,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E67" t="s">
         <v>9</v>
       </c>
@@ -1329,7 +1345,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B68">
         <v>10</v>
       </c>
@@ -1343,7 +1359,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H69" t="s">
         <v>9</v>
       </c>
@@ -1351,7 +1367,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B70">
         <v>2</v>
       </c>
@@ -1365,7 +1381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E71" t="s">
         <v>9</v>
       </c>
@@ -1373,7 +1389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B72">
         <v>15</v>
       </c>
@@ -1389,6 +1405,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update after the first 4 games completed
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D805A157-9AE0-43CE-B6BC-31C4601DBDF0}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497F10AE-9233-4334-BDC0-E19775124DA4}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -307,6 +307,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -775,6 +779,9 @@
       <c r="C15" t="s">
         <v>16</v>
       </c>
+      <c r="AK15">
+        <v>82</v>
+      </c>
       <c r="AL15" t="s">
         <v>17</v>
       </c>
@@ -787,7 +794,7 @@
         <v>9</v>
       </c>
       <c r="AJ16" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -797,6 +804,9 @@
       <c r="C17" t="s">
         <v>18</v>
       </c>
+      <c r="AK17">
+        <v>83</v>
+      </c>
       <c r="AL17" t="s">
         <v>19</v>
       </c>
@@ -872,6 +882,9 @@
       <c r="C23" t="s">
         <v>26</v>
       </c>
+      <c r="D23">
+        <v>83</v>
+      </c>
       <c r="AL23" t="s">
         <v>27</v>
       </c>
@@ -881,7 +894,7 @@
     </row>
     <row r="24" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="AJ24" t="s">
         <v>9</v>
@@ -894,6 +907,9 @@
       <c r="C25" t="s">
         <v>28</v>
       </c>
+      <c r="D25">
+        <v>79</v>
+      </c>
       <c r="AL25" t="s">
         <v>29</v>
       </c>
@@ -1189,6 +1205,9 @@
       <c r="C54" t="s">
         <v>56</v>
       </c>
+      <c r="D54">
+        <v>76</v>
+      </c>
       <c r="R54" t="s">
         <v>57</v>
       </c>
@@ -1201,7 +1220,7 @@
     </row>
     <row r="55" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E55" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="AJ55" t="s">
         <v>9</v>
@@ -1213,6 +1232,9 @@
       </c>
       <c r="C56" t="s">
         <v>59</v>
+      </c>
+      <c r="D56">
+        <v>47</v>
       </c>
       <c r="AL56" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
updated for evening games
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497F10AE-9233-4334-BDC0-E19775124DA4}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{656A7C40-B26C-496D-8556-4E6CEC7E43DC}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -685,6 +685,9 @@
       <c r="C7" t="s">
         <v>7</v>
       </c>
+      <c r="D7">
+        <v>71</v>
+      </c>
       <c r="AL7" t="s">
         <v>8</v>
       </c>
@@ -694,7 +697,7 @@
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AJ8" t="s">
         <v>9</v>
@@ -707,6 +710,9 @@
       <c r="C9" t="s">
         <v>10</v>
       </c>
+      <c r="D9">
+        <v>65</v>
+      </c>
       <c r="AL9" t="s">
         <v>11</v>
       </c>
@@ -832,6 +838,9 @@
       <c r="P19" t="s">
         <v>79</v>
       </c>
+      <c r="AK19">
+        <v>97</v>
+      </c>
       <c r="AL19" t="s">
         <v>21</v>
       </c>
@@ -844,7 +853,7 @@
         <v>9</v>
       </c>
       <c r="AJ20" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -854,6 +863,9 @@
       <c r="C21" t="s">
         <v>22</v>
       </c>
+      <c r="AK21">
+        <v>78</v>
+      </c>
       <c r="AL21" t="s">
         <v>23</v>
       </c>
@@ -932,6 +944,9 @@
       <c r="C27" t="s">
         <v>30</v>
       </c>
+      <c r="D27">
+        <v>92</v>
+      </c>
       <c r="AL27" t="s">
         <v>31</v>
       </c>
@@ -941,7 +956,7 @@
     </row>
     <row r="28" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E28" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="AJ28" t="s">
         <v>9</v>
@@ -954,6 +969,9 @@
       <c r="C29" t="s">
         <v>32</v>
       </c>
+      <c r="D29">
+        <v>67</v>
+      </c>
       <c r="AL29" t="s">
         <v>33</v>
       </c>
@@ -1158,6 +1176,9 @@
       <c r="C50" t="s">
         <v>51</v>
       </c>
+      <c r="D50">
+        <v>78</v>
+      </c>
       <c r="S50" t="s">
         <v>52</v>
       </c>
@@ -1170,7 +1191,7 @@
     </row>
     <row r="51" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E51" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="AJ51" t="s">
         <v>9</v>
@@ -1182,6 +1203,9 @@
       </c>
       <c r="C52" t="s">
         <v>54</v>
+      </c>
+      <c r="D52">
+        <v>68</v>
       </c>
       <c r="AL52" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
updae for recent matches, march and crokinole
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{656A7C40-B26C-496D-8556-4E6CEC7E43DC}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA2214A8-E025-436F-9E6C-14D9110BFF6E}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="81">
   <si>
     <t>2026 March Madness Bracket</t>
   </si>
@@ -255,6 +255,9 @@
   </si>
   <si>
     <t>s</t>
+  </si>
+  <si>
+    <t>Texas</t>
   </si>
 </sst>
 </file>
@@ -897,6 +900,9 @@
       <c r="D23">
         <v>83</v>
       </c>
+      <c r="AK23">
+        <v>71</v>
+      </c>
       <c r="AL23" t="s">
         <v>27</v>
       </c>
@@ -909,7 +915,7 @@
         <v>26</v>
       </c>
       <c r="AJ24" t="s">
-        <v>9</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -922,6 +928,9 @@
       <c r="D25">
         <v>79</v>
       </c>
+      <c r="AK25">
+        <v>79</v>
+      </c>
       <c r="AL25" t="s">
         <v>29</v>
       </c>
@@ -1082,6 +1091,9 @@
       <c r="C42" t="s">
         <v>42</v>
       </c>
+      <c r="AK42">
+        <v>101</v>
+      </c>
       <c r="AL42" t="s">
         <v>43</v>
       </c>
@@ -1094,7 +1106,7 @@
         <v>9</v>
       </c>
       <c r="AJ43" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1107,6 +1119,9 @@
       <c r="R44" t="s">
         <v>9</v>
       </c>
+      <c r="AK44">
+        <v>80</v>
+      </c>
       <c r="AL44" t="s">
         <v>45</v>
       </c>
@@ -1288,6 +1303,9 @@
       <c r="C58" t="s">
         <v>63</v>
       </c>
+      <c r="D58">
+        <v>78</v>
+      </c>
       <c r="AL58" t="s">
         <v>64</v>
       </c>
@@ -1297,7 +1315,7 @@
     </row>
     <row r="59" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E59" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="AJ59" t="s">
         <v>9</v>
@@ -1310,6 +1328,9 @@
       <c r="C60" t="s">
         <v>65</v>
       </c>
+      <c r="D60">
+        <v>82</v>
+      </c>
       <c r="AL60" t="s">
         <v>66</v>
       </c>
@@ -1376,6 +1397,9 @@
       <c r="C66" t="s">
         <v>71</v>
       </c>
+      <c r="D66">
+        <v>50</v>
+      </c>
       <c r="AL66" t="s">
         <v>72</v>
       </c>
@@ -1385,7 +1409,7 @@
     </row>
     <row r="67" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E67" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="AJ67" t="s">
         <v>9</v>
@@ -1397,6 +1421,9 @@
       </c>
       <c r="C68" t="s">
         <v>73</v>
+      </c>
+      <c r="D68">
+        <v>63</v>
       </c>
       <c r="AL68" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
updated for last games of the day
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B2B6F52-431D-40D2-814B-BD568F426C85}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39B74BA1-0F32-44D1-9770-87A5F0685979}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -965,7 +965,7 @@
         <v>30</v>
       </c>
       <c r="AJ28" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1156,7 +1156,7 @@
         <v>9</v>
       </c>
       <c r="AJ47" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1350,6 +1350,9 @@
       <c r="C62" t="s">
         <v>67</v>
       </c>
+      <c r="D62">
+        <v>105</v>
+      </c>
       <c r="AL62" t="s">
         <v>68</v>
       </c>
@@ -1359,7 +1362,7 @@
     </row>
     <row r="63" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E63" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="AJ63" t="s">
         <v>9</v>
@@ -1372,6 +1375,9 @@
       <c r="C64" t="s">
         <v>69</v>
       </c>
+      <c r="D64">
+        <v>70</v>
+      </c>
       <c r="AL64" t="s">
         <v>70</v>
       </c>
@@ -1453,7 +1459,7 @@
     </row>
     <row r="71" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E71" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="AJ71" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
updated for most recent games and some visual changes
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="51" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39B74BA1-0F32-44D1-9770-87A5F0685979}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E4D3A29-D70F-42A0-B419-D84146D8A3D2}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="79">
   <si>
     <t>2026 March Madness Bracket</t>
   </si>
@@ -252,9 +252,6 @@
   </si>
   <si>
     <t>Tennessee State</t>
-  </si>
-  <si>
-    <t>s</t>
   </si>
 </sst>
 </file>
@@ -688,6 +685,9 @@
       <c r="D7">
         <v>71</v>
       </c>
+      <c r="AK7">
+        <v>92</v>
+      </c>
       <c r="AL7" t="s">
         <v>8</v>
       </c>
@@ -700,7 +700,7 @@
         <v>7</v>
       </c>
       <c r="AJ8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.55000000000000004">
@@ -713,6 +713,9 @@
       <c r="D9">
         <v>65</v>
       </c>
+      <c r="AK9">
+        <v>58</v>
+      </c>
       <c r="AL9" t="s">
         <v>11</v>
       </c>
@@ -738,6 +741,9 @@
       <c r="D11">
         <v>64</v>
       </c>
+      <c r="AK11">
+        <v>76</v>
+      </c>
       <c r="AL11" t="s">
         <v>13</v>
       </c>
@@ -750,7 +756,7 @@
         <v>14</v>
       </c>
       <c r="AJ12" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.55000000000000004">
@@ -762,6 +768,9 @@
       </c>
       <c r="D13">
         <v>66</v>
+      </c>
+      <c r="AK13">
+        <v>86</v>
       </c>
       <c r="AL13" t="s">
         <v>15</v>
@@ -785,6 +794,9 @@
       <c r="C15" t="s">
         <v>16</v>
       </c>
+      <c r="D15">
+        <v>79</v>
+      </c>
       <c r="AK15">
         <v>82</v>
       </c>
@@ -797,7 +809,7 @@
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E16" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AJ16" t="s">
         <v>19</v>
@@ -810,6 +822,9 @@
       <c r="C17" t="s">
         <v>18</v>
       </c>
+      <c r="D17">
+        <v>53</v>
+      </c>
       <c r="AK17">
         <v>83</v>
       </c>
@@ -835,8 +850,8 @@
       <c r="C19" t="s">
         <v>20</v>
       </c>
-      <c r="P19" t="s">
-        <v>79</v>
+      <c r="D19">
+        <v>68</v>
       </c>
       <c r="AK19">
         <v>97</v>
@@ -850,7 +865,7 @@
     </row>
     <row r="20" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E20" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="AJ20" t="s">
         <v>21</v>
@@ -863,6 +878,9 @@
       <c r="C21" t="s">
         <v>22</v>
       </c>
+      <c r="D21">
+        <v>60</v>
+      </c>
       <c r="AK21">
         <v>78</v>
       </c>
@@ -953,6 +971,9 @@
       <c r="D27">
         <v>92</v>
       </c>
+      <c r="AK27">
+        <v>73</v>
+      </c>
       <c r="AL27" t="s">
         <v>31</v>
       </c>
@@ -978,6 +999,9 @@
       <c r="D29">
         <v>67</v>
       </c>
+      <c r="AK29">
+        <v>64</v>
+      </c>
       <c r="AL29" t="s">
         <v>33</v>
       </c>
@@ -1000,6 +1024,12 @@
       <c r="C31" t="s">
         <v>34</v>
       </c>
+      <c r="D31">
+        <v>75</v>
+      </c>
+      <c r="AK31">
+        <v>80</v>
+      </c>
       <c r="AL31" t="s">
         <v>35</v>
       </c>
@@ -1009,10 +1039,10 @@
     </row>
     <row r="32" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E32" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="AJ32" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1022,6 +1052,12 @@
       <c r="C33" t="s">
         <v>36</v>
       </c>
+      <c r="D33">
+        <v>71</v>
+      </c>
+      <c r="AK33">
+        <v>66</v>
+      </c>
       <c r="AL33" t="s">
         <v>37</v>
       </c>
@@ -1044,6 +1080,12 @@
       <c r="C35" t="s">
         <v>38</v>
       </c>
+      <c r="D35">
+        <v>82</v>
+      </c>
+      <c r="AK35">
+        <v>104</v>
+      </c>
       <c r="AL35" t="s">
         <v>39</v>
       </c>
@@ -1053,10 +1095,10 @@
     </row>
     <row r="36" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E36" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="AJ36" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1066,6 +1108,12 @@
       <c r="C37" t="s">
         <v>40</v>
       </c>
+      <c r="D37">
+        <v>71</v>
+      </c>
+      <c r="AK37">
+        <v>71</v>
+      </c>
       <c r="AL37" t="s">
         <v>41</v>
       </c>
@@ -1088,6 +1136,9 @@
       <c r="C42" t="s">
         <v>42</v>
       </c>
+      <c r="D42">
+        <v>114</v>
+      </c>
       <c r="AK42">
         <v>101</v>
       </c>
@@ -1100,7 +1151,7 @@
     </row>
     <row r="43" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E43" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="AJ43" t="s">
         <v>43</v>
@@ -1113,6 +1164,9 @@
       <c r="C44" t="s">
         <v>44</v>
       </c>
+      <c r="D44">
+        <v>55</v>
+      </c>
       <c r="R44" t="s">
         <v>9</v>
       </c>
@@ -1141,9 +1195,15 @@
       <c r="C46" t="s">
         <v>46</v>
       </c>
+      <c r="D46">
+        <v>61</v>
+      </c>
       <c r="R46" t="s">
         <v>47</v>
       </c>
+      <c r="AK46">
+        <v>77</v>
+      </c>
       <c r="AL46" t="s">
         <v>48</v>
       </c>
@@ -1153,7 +1213,7 @@
     </row>
     <row r="47" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E47" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="AJ47" t="s">
         <v>50</v>
@@ -1165,6 +1225,12 @@
       </c>
       <c r="C48" t="s">
         <v>49</v>
+      </c>
+      <c r="D48">
+        <v>67</v>
+      </c>
+      <c r="AK48">
+        <v>102</v>
       </c>
       <c r="AL48" t="s">
         <v>50</v>
@@ -1194,6 +1260,9 @@
       <c r="S50" t="s">
         <v>52</v>
       </c>
+      <c r="AK50">
+        <v>91</v>
+      </c>
       <c r="AL50" t="s">
         <v>53</v>
       </c>
@@ -1206,7 +1275,7 @@
         <v>51</v>
       </c>
       <c r="AJ51" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
     </row>
     <row r="52" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1219,6 +1288,9 @@
       <c r="D52">
         <v>68</v>
       </c>
+      <c r="AK52">
+        <v>71</v>
+      </c>
       <c r="AL52" t="s">
         <v>55</v>
       </c>
@@ -1247,6 +1319,9 @@
       <c r="R54" t="s">
         <v>57</v>
       </c>
+      <c r="AK54">
+        <v>90</v>
+      </c>
       <c r="AL54" t="s">
         <v>58</v>
       </c>
@@ -1259,7 +1334,7 @@
         <v>56</v>
       </c>
       <c r="AJ55" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1272,6 +1347,9 @@
       <c r="D56">
         <v>47</v>
       </c>
+      <c r="AK56">
+        <v>70</v>
+      </c>
       <c r="AL56" t="s">
         <v>60</v>
       </c>
@@ -1303,6 +1381,9 @@
       <c r="D58">
         <v>78</v>
       </c>
+      <c r="AK58">
+        <v>78</v>
+      </c>
       <c r="AL58" t="s">
         <v>64</v>
       </c>
@@ -1315,7 +1396,7 @@
         <v>65</v>
       </c>
       <c r="AJ59" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
     </row>
     <row r="60" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1328,6 +1409,9 @@
       <c r="D60">
         <v>82</v>
       </c>
+      <c r="AK60">
+        <v>56</v>
+      </c>
       <c r="AL60" t="s">
         <v>66</v>
       </c>
@@ -1353,6 +1437,9 @@
       <c r="D62">
         <v>105</v>
       </c>
+      <c r="AK62">
+        <v>82</v>
+      </c>
       <c r="AL62" t="s">
         <v>68</v>
       </c>
@@ -1365,7 +1452,7 @@
         <v>67</v>
       </c>
       <c r="AJ63" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1378,6 +1465,9 @@
       <c r="D64">
         <v>70</v>
       </c>
+      <c r="AK64">
+        <v>73</v>
+      </c>
       <c r="AL64" t="s">
         <v>70</v>
       </c>
@@ -1403,6 +1493,9 @@
       <c r="D66">
         <v>50</v>
       </c>
+      <c r="AK66">
+        <v>89</v>
+      </c>
       <c r="AL66" t="s">
         <v>72</v>
       </c>
@@ -1415,7 +1508,7 @@
         <v>73</v>
       </c>
       <c r="AJ67" t="s">
-        <v>9</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1428,6 +1521,9 @@
       <c r="D68">
         <v>63</v>
       </c>
+      <c r="AK68">
+        <v>84</v>
+      </c>
       <c r="AL68" t="s">
         <v>74</v>
       </c>
@@ -1450,6 +1546,12 @@
       <c r="C70" t="s">
         <v>75</v>
       </c>
+      <c r="D70">
+        <v>78</v>
+      </c>
+      <c r="AK70">
+        <v>108</v>
+      </c>
       <c r="AL70" t="s">
         <v>76</v>
       </c>
@@ -1462,7 +1564,7 @@
         <v>75</v>
       </c>
       <c r="AJ71" t="s">
-        <v>9</v>
+        <v>76</v>
       </c>
     </row>
     <row r="72" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1471,6 +1573,12 @@
       </c>
       <c r="C72" t="s">
         <v>77</v>
+      </c>
+      <c r="D72">
+        <v>47</v>
+      </c>
+      <c r="AK72">
+        <v>74</v>
       </c>
       <c r="AL72" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
updated after texas game
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="108" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E4D3A29-D70F-42A0-B419-D84146D8A3D2}"/>
+  <xr:revisionPtr revIDLastSave="128" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{669522F5-88E2-45E5-B65E-292F219801A4}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -699,6 +699,9 @@
       <c r="E8" t="s">
         <v>7</v>
       </c>
+      <c r="F8">
+        <v>81</v>
+      </c>
       <c r="AJ8" t="s">
         <v>8</v>
       </c>
@@ -725,7 +728,7 @@
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AG10" t="s">
         <v>9</v>
@@ -755,6 +758,9 @@
       <c r="E12" t="s">
         <v>14</v>
       </c>
+      <c r="F12">
+        <v>58</v>
+      </c>
       <c r="AJ12" t="s">
         <v>15</v>
       </c>
@@ -929,6 +935,12 @@
       <c r="E24" t="s">
         <v>26</v>
       </c>
+      <c r="F24">
+        <v>69</v>
+      </c>
+      <c r="AI24">
+        <v>74</v>
+      </c>
       <c r="AJ24" t="s">
         <v>29</v>
       </c>
@@ -955,10 +967,10 @@
     </row>
     <row r="26" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H26" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="AG26" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -985,6 +997,12 @@
       <c r="E28" t="s">
         <v>30</v>
       </c>
+      <c r="F28">
+        <v>77</v>
+      </c>
+      <c r="AI28">
+        <v>68</v>
+      </c>
       <c r="AJ28" t="s">
         <v>31</v>
       </c>
@@ -1153,6 +1171,9 @@
       <c r="E43" t="s">
         <v>42</v>
       </c>
+      <c r="AI43">
+        <v>95</v>
+      </c>
       <c r="AJ43" t="s">
         <v>43</v>
       </c>
@@ -1185,7 +1206,7 @@
         <v>9</v>
       </c>
       <c r="AG45" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1215,6 +1236,9 @@
       <c r="E47" t="s">
         <v>49</v>
       </c>
+      <c r="AI47">
+        <v>72</v>
+      </c>
       <c r="AJ47" t="s">
         <v>50</v>
       </c>
@@ -1507,6 +1531,9 @@
       <c r="E67" t="s">
         <v>73</v>
       </c>
+      <c r="F67">
+        <v>57</v>
+      </c>
       <c r="AJ67" t="s">
         <v>72</v>
       </c>
@@ -1533,7 +1560,7 @@
     </row>
     <row r="69" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H69" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="AG69" t="s">
         <v>9</v>
@@ -1562,6 +1589,9 @@
     <row r="71" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E71" t="s">
         <v>75</v>
+      </c>
+      <c r="F71">
+        <v>88</v>
       </c>
       <c r="AJ71" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
updated for last of 3 22 games
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="128" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{669522F5-88E2-45E5-B65E-292F219801A4}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49AC669F-C783-456F-B988-EC4CBD2A8516}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -817,6 +817,9 @@
       <c r="E16" t="s">
         <v>16</v>
       </c>
+      <c r="AI16">
+        <v>88</v>
+      </c>
       <c r="AJ16" t="s">
         <v>19</v>
       </c>
@@ -846,7 +849,7 @@
         <v>9</v>
       </c>
       <c r="AG18" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -873,6 +876,9 @@
       <c r="E20" t="s">
         <v>20</v>
       </c>
+      <c r="AI20">
+        <v>94</v>
+      </c>
       <c r="AJ20" t="s">
         <v>21</v>
       </c>
@@ -1298,6 +1304,9 @@
       <c r="E51" t="s">
         <v>51</v>
       </c>
+      <c r="F51">
+        <v>72</v>
+      </c>
       <c r="AJ51" t="s">
         <v>53</v>
       </c>
@@ -1324,7 +1333,7 @@
     </row>
     <row r="53" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H53" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="AG53" t="s">
         <v>9</v>
@@ -1357,6 +1366,9 @@
       <c r="E55" t="s">
         <v>56</v>
       </c>
+      <c r="F55">
+        <v>74</v>
+      </c>
       <c r="AJ55" t="s">
         <v>58</v>
       </c>
@@ -1419,6 +1431,9 @@
       <c r="E59" t="s">
         <v>65</v>
       </c>
+      <c r="F59">
+        <v>55</v>
+      </c>
       <c r="AJ59" t="s">
         <v>64</v>
       </c>
@@ -1445,7 +1460,7 @@
     </row>
     <row r="61" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H61" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="AG61" t="s">
         <v>9</v>
@@ -1474,6 +1489,9 @@
     <row r="63" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E63" t="s">
         <v>67</v>
+      </c>
+      <c r="F63">
+        <v>76</v>
       </c>
       <c r="AJ63" t="s">
         <v>68</v>

</xml_diff>

<commit_message>
updated for live games
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="137" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49AC669F-C783-456F-B988-EC4CBD2A8516}"/>
+  <xr:revisionPtr revIDLastSave="147" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9AD1D45-E740-4725-B538-EC9B64F5C2C4}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -817,6 +817,9 @@
       <c r="E16" t="s">
         <v>16</v>
       </c>
+      <c r="F16">
+        <v>67</v>
+      </c>
       <c r="AI16">
         <v>88</v>
       </c>
@@ -846,7 +849,7 @@
     </row>
     <row r="18" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H18" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="AG18" t="s">
         <v>21</v>
@@ -876,6 +879,9 @@
       <c r="E20" t="s">
         <v>20</v>
       </c>
+      <c r="F20">
+        <v>65</v>
+      </c>
       <c r="AI20">
         <v>94</v>
       </c>
@@ -1065,6 +1071,9 @@
       <c r="E32" t="s">
         <v>34</v>
       </c>
+      <c r="AI32">
+        <v>69</v>
+      </c>
       <c r="AJ32" t="s">
         <v>35</v>
       </c>
@@ -1094,7 +1103,7 @@
         <v>9</v>
       </c>
       <c r="AG34" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1121,6 +1130,9 @@
       <c r="E36" t="s">
         <v>38</v>
       </c>
+      <c r="AI36">
+        <v>79</v>
+      </c>
       <c r="AJ36" t="s">
         <v>39</v>
       </c>
@@ -1552,6 +1564,9 @@
       <c r="F67">
         <v>57</v>
       </c>
+      <c r="AI67">
+        <v>63</v>
+      </c>
       <c r="AJ67" t="s">
         <v>72</v>
       </c>
@@ -1581,7 +1596,7 @@
         <v>75</v>
       </c>
       <c r="AG69" t="s">
-        <v>9</v>
+        <v>76</v>
       </c>
     </row>
     <row r="70" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1610,6 +1625,9 @@
       </c>
       <c r="F71">
         <v>88</v>
+      </c>
+      <c r="AI71">
+        <v>82</v>
       </c>
       <c r="AJ71" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
updated after florida game
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="147" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9AD1D45-E740-4725-B538-EC9B64F5C2C4}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB8F5431-0573-44CE-8932-A8EA899BE9E2}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -702,6 +702,9 @@
       <c r="F8">
         <v>81</v>
       </c>
+      <c r="AI8">
+        <v>78</v>
+      </c>
       <c r="AJ8" t="s">
         <v>8</v>
       </c>
@@ -731,7 +734,7 @@
         <v>7</v>
       </c>
       <c r="AG10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.55000000000000004">
@@ -761,6 +764,9 @@
       <c r="F12">
         <v>58</v>
       </c>
+      <c r="AI12">
+        <v>66</v>
+      </c>
       <c r="AJ12" t="s">
         <v>15</v>
       </c>
@@ -1189,6 +1195,9 @@
       <c r="E43" t="s">
         <v>42</v>
       </c>
+      <c r="F43">
+        <v>72</v>
+      </c>
       <c r="AI43">
         <v>95</v>
       </c>
@@ -1221,7 +1230,7 @@
     </row>
     <row r="45" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H45" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="AG45" t="s">
         <v>43</v>
@@ -1254,6 +1263,9 @@
       <c r="E47" t="s">
         <v>49</v>
       </c>
+      <c r="F47">
+        <v>73</v>
+      </c>
       <c r="AI47">
         <v>72</v>
       </c>
@@ -1446,6 +1458,9 @@
       <c r="F59">
         <v>55</v>
       </c>
+      <c r="AI59">
+        <v>79</v>
+      </c>
       <c r="AJ59" t="s">
         <v>64</v>
       </c>
@@ -1475,7 +1490,7 @@
         <v>67</v>
       </c>
       <c r="AG61" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1504,6 +1519,9 @@
       </c>
       <c r="F63">
         <v>76</v>
+      </c>
+      <c r="AI63">
+        <v>72</v>
       </c>
       <c r="AJ63" t="s">
         <v>68</v>

</xml_diff>

<commit_message>
upadated with newest results
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="157" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB8F5431-0573-44CE-8932-A8EA899BE9E2}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{984CADE3-676E-4FE1-89D9-76C600700735}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1077,6 +1077,9 @@
       <c r="E32" t="s">
         <v>34</v>
       </c>
+      <c r="F32">
+        <v>57</v>
+      </c>
       <c r="AI32">
         <v>69</v>
       </c>
@@ -1106,7 +1109,7 @@
     </row>
     <row r="34" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H34" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="AG34" t="s">
         <v>39</v>
@@ -1136,6 +1139,9 @@
       <c r="E36" t="s">
         <v>38</v>
       </c>
+      <c r="F36">
+        <v>73</v>
+      </c>
       <c r="AI36">
         <v>79</v>
       </c>
@@ -1331,6 +1337,9 @@
       <c r="F51">
         <v>72</v>
       </c>
+      <c r="AI51">
+        <v>65</v>
+      </c>
       <c r="AJ51" t="s">
         <v>53</v>
       </c>
@@ -1360,7 +1369,7 @@
         <v>56</v>
       </c>
       <c r="AG53" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="54" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1392,6 +1401,9 @@
       </c>
       <c r="F55">
         <v>74</v>
+      </c>
+      <c r="AI55">
+        <v>90</v>
       </c>
       <c r="AJ55" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
updated odds for the rest of tonights games
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="172" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1233BC58-E4CF-4B08-B5AB-1EFCADB021C9}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBCAD54B-30D0-4386-BC24-F9ABEAAC8EDF}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,6 +733,9 @@
       <c r="H10" t="s">
         <v>7</v>
       </c>
+      <c r="AF10">
+        <v>109</v>
+      </c>
       <c r="AG10" t="s">
         <v>8</v>
       </c>
@@ -796,7 +799,7 @@
         <v>9</v>
       </c>
       <c r="AD14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.55000000000000004">
@@ -857,6 +860,9 @@
       <c r="H18" t="s">
         <v>16</v>
       </c>
+      <c r="AF18">
+        <v>88</v>
+      </c>
       <c r="AG18" t="s">
         <v>21</v>
       </c>
@@ -1513,6 +1519,9 @@
       <c r="H61" t="s">
         <v>67</v>
       </c>
+      <c r="I61">
+        <v>65</v>
+      </c>
       <c r="AG61" t="s">
         <v>64</v>
       </c>
@@ -1573,7 +1582,7 @@
     </row>
     <row r="65" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K65" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="AD65" t="s">
         <v>9</v>
@@ -1636,6 +1645,9 @@
     <row r="69" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H69" t="s">
         <v>75</v>
+      </c>
+      <c r="I69">
+        <v>55</v>
       </c>
       <c r="AG69" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
updated for most recent round
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="181" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBCAD54B-30D0-4386-BC24-F9ABEAAC8EDF}"/>
+  <xr:revisionPtr revIDLastSave="193" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA3F982-E3DB-41C8-8B0E-4218657A6CC2}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,6 +733,9 @@
       <c r="H10" t="s">
         <v>7</v>
       </c>
+      <c r="I10">
+        <v>80</v>
+      </c>
       <c r="AF10">
         <v>109</v>
       </c>
@@ -796,7 +799,7 @@
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K14" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD14" t="s">
         <v>8</v>
@@ -860,6 +863,9 @@
       <c r="H18" t="s">
         <v>16</v>
       </c>
+      <c r="I18">
+        <v>75</v>
+      </c>
       <c r="AF18">
         <v>88</v>
       </c>
@@ -993,6 +999,9 @@
       <c r="H26" t="s">
         <v>30</v>
       </c>
+      <c r="I26">
+        <v>63</v>
+      </c>
       <c r="AF26">
         <v>77</v>
       </c>
@@ -1056,7 +1065,7 @@
     </row>
     <row r="30" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K30" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="AD30" t="s">
         <v>39</v>
@@ -1120,6 +1129,9 @@
       <c r="H34" t="s">
         <v>38</v>
       </c>
+      <c r="I34">
+        <v>67</v>
+      </c>
       <c r="AF34">
         <v>79</v>
       </c>
@@ -1253,6 +1265,9 @@
       <c r="I45">
         <v>77</v>
       </c>
+      <c r="AF45">
+        <v>90</v>
+      </c>
       <c r="AG45" t="s">
         <v>43</v>
       </c>
@@ -1319,7 +1334,7 @@
         <v>49</v>
       </c>
       <c r="AD49" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1386,6 +1401,9 @@
       <c r="I53">
         <v>71</v>
       </c>
+      <c r="AF53">
+        <v>77</v>
+      </c>
       <c r="AG53" t="s">
         <v>58</v>
       </c>
@@ -1522,6 +1540,9 @@
       <c r="I61">
         <v>65</v>
       </c>
+      <c r="AF61">
+        <v>76</v>
+      </c>
       <c r="AG61" t="s">
         <v>64</v>
       </c>
@@ -1585,7 +1606,7 @@
         <v>67</v>
       </c>
       <c r="AD65" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1648,6 +1669,9 @@
       </c>
       <c r="I69">
         <v>55</v>
+      </c>
+      <c r="AF69">
+        <v>62</v>
       </c>
       <c r="AG69" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
update for first round of elite 8 games
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="193" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA3F982-E3DB-41C8-8B0E-4218657A6CC2}"/>
+  <xr:revisionPtr revIDLastSave="201" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D2844BE-6DBF-46C7-8424-FF1B517B8EE0}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -801,6 +801,9 @@
       <c r="K14" t="s">
         <v>7</v>
       </c>
+      <c r="AC14">
+        <v>79</v>
+      </c>
       <c r="AD14" t="s">
         <v>8</v>
       </c>
@@ -935,7 +938,7 @@
         <v>9</v>
       </c>
       <c r="AA22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AD22" t="s">
         <v>25</v>
@@ -1067,6 +1070,9 @@
       <c r="K30" t="s">
         <v>38</v>
       </c>
+      <c r="AC30">
+        <v>64</v>
+      </c>
       <c r="AD30" t="s">
         <v>39</v>
       </c>
@@ -1333,6 +1339,9 @@
       <c r="K49" t="s">
         <v>49</v>
       </c>
+      <c r="L49">
+        <v>59</v>
+      </c>
       <c r="AD49" t="s">
         <v>43</v>
       </c>
@@ -1470,7 +1479,7 @@
         <v>61</v>
       </c>
       <c r="N57" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="AA57" t="s">
         <v>9</v>
@@ -1604,6 +1613,9 @@
     <row r="65" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K65" t="s">
         <v>67</v>
+      </c>
+      <c r="L65">
+        <v>71</v>
       </c>
       <c r="AD65" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
updated for rest of elite 8
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,14 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="201" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D2844BE-6DBF-46C7-8424-FF1B517B8EE0}"/>
+  <xr:revisionPtr revIDLastSave="207" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F21794E-505B-477E-A10C-E80EC5E2A80B}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="madness" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -801,6 +814,9 @@
       <c r="K14" t="s">
         <v>7</v>
       </c>
+      <c r="L14">
+        <v>72</v>
+      </c>
       <c r="AC14">
         <v>79</v>
       </c>
@@ -935,7 +951,7 @@
         <v>24</v>
       </c>
       <c r="N22" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="AA22" t="s">
         <v>8</v>
@@ -1070,6 +1086,9 @@
       <c r="K30" t="s">
         <v>38</v>
       </c>
+      <c r="L30">
+        <v>73</v>
+      </c>
       <c r="AC30">
         <v>64</v>
       </c>
@@ -1342,6 +1361,9 @@
       <c r="L49">
         <v>59</v>
       </c>
+      <c r="AC49">
+        <v>95</v>
+      </c>
       <c r="AD49" t="s">
         <v>43</v>
       </c>
@@ -1482,7 +1504,7 @@
         <v>67</v>
       </c>
       <c r="AA57" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="AD57" t="s">
         <v>62</v>
@@ -1616,6 +1638,9 @@
       </c>
       <c r="L65">
         <v>71</v>
+      </c>
+      <c r="AC65">
+        <v>62</v>
       </c>
       <c r="AD65" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
added pizza bracket and updated final march madness
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
+++ b/static/marchMadness/2026/results-bracket-march-madness-2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="216" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CF80B4C-39DB-4DA3-B8B1-B319223F86B1}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="11_1E2582D9B22B9E23A05D16462BA71CED684F7CDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D994E6DB-D973-4C7C-9AF6-047849874037}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="78">
   <si>
     <t>2026 March Madness Bracket</t>
   </si>
@@ -55,9 +55,6 @@
   </si>
   <si>
     <t>Arizona</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Siena</t>
@@ -727,7 +724,7 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9">
         <v>65</v>
@@ -736,7 +733,7 @@
         <v>58</v>
       </c>
       <c r="AL9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AM9">
         <v>16</v>
@@ -761,7 +758,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11">
         <v>64</v>
@@ -770,7 +767,7 @@
         <v>76</v>
       </c>
       <c r="AL11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AM11">
         <v>8</v>
@@ -778,7 +775,7 @@
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12">
         <v>58</v>
@@ -787,7 +784,7 @@
         <v>66</v>
       </c>
       <c r="AJ12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.55000000000000004">
@@ -795,7 +792,7 @@
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13">
         <v>66</v>
@@ -804,7 +801,7 @@
         <v>86</v>
       </c>
       <c r="AL13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AM13">
         <v>9</v>
@@ -829,7 +826,7 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>79</v>
@@ -838,7 +835,7 @@
         <v>82</v>
       </c>
       <c r="AL15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AM15">
         <v>5</v>
@@ -846,7 +843,7 @@
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F16">
         <v>67</v>
@@ -855,7 +852,7 @@
         <v>88</v>
       </c>
       <c r="AJ16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -863,7 +860,7 @@
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>53</v>
@@ -872,7 +869,7 @@
         <v>83</v>
       </c>
       <c r="AL17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM17">
         <v>12</v>
@@ -880,7 +877,7 @@
     </row>
     <row r="18" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I18">
         <v>75</v>
@@ -889,7 +886,7 @@
         <v>88</v>
       </c>
       <c r="AG18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -897,7 +894,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19">
         <v>68</v>
@@ -906,7 +903,7 @@
         <v>97</v>
       </c>
       <c r="AL19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AM19">
         <v>4</v>
@@ -914,7 +911,7 @@
     </row>
     <row r="20" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20">
         <v>65</v>
@@ -923,7 +920,7 @@
         <v>94</v>
       </c>
       <c r="AJ20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -931,7 +928,7 @@
         <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21">
         <v>60</v>
@@ -940,7 +937,7 @@
         <v>78</v>
       </c>
       <c r="AL21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AM21">
         <v>13</v>
@@ -948,10 +945,10 @@
     </row>
     <row r="22" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O22">
         <v>71</v>
@@ -963,7 +960,7 @@
         <v>8</v>
       </c>
       <c r="AD22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -971,7 +968,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D23">
         <v>83</v>
@@ -980,7 +977,7 @@
         <v>71</v>
       </c>
       <c r="AL23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AM23">
         <v>6</v>
@@ -988,7 +985,7 @@
     </row>
     <row r="24" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F24">
         <v>69</v>
@@ -997,7 +994,7 @@
         <v>74</v>
       </c>
       <c r="AJ24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1005,7 +1002,7 @@
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D25">
         <v>79</v>
@@ -1014,7 +1011,7 @@
         <v>79</v>
       </c>
       <c r="AL25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AM25">
         <v>11</v>
@@ -1022,7 +1019,7 @@
     </row>
     <row r="26" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I26">
         <v>63</v>
@@ -1031,7 +1028,7 @@
         <v>77</v>
       </c>
       <c r="AG26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1039,7 +1036,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D27">
         <v>92</v>
@@ -1048,7 +1045,7 @@
         <v>73</v>
       </c>
       <c r="AL27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AM27">
         <v>3</v>
@@ -1056,7 +1053,7 @@
     </row>
     <row r="28" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F28">
         <v>77</v>
@@ -1065,7 +1062,7 @@
         <v>68</v>
       </c>
       <c r="AJ28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1073,7 +1070,7 @@
         <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D29">
         <v>67</v>
@@ -1082,7 +1079,7 @@
         <v>64</v>
       </c>
       <c r="AL29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AM29">
         <v>14</v>
@@ -1090,7 +1087,7 @@
     </row>
     <row r="30" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L30">
         <v>73</v>
@@ -1099,7 +1096,7 @@
         <v>64</v>
       </c>
       <c r="AD30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1107,7 +1104,7 @@
         <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D31">
         <v>75</v>
@@ -1116,7 +1113,7 @@
         <v>80</v>
       </c>
       <c r="AL31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AM31">
         <v>7</v>
@@ -1124,7 +1121,7 @@
     </row>
     <row r="32" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F32">
         <v>57</v>
@@ -1133,7 +1130,7 @@
         <v>69</v>
       </c>
       <c r="AJ32" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1141,7 +1138,7 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D33">
         <v>71</v>
@@ -1150,7 +1147,7 @@
         <v>66</v>
       </c>
       <c r="AL33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AM33">
         <v>10</v>
@@ -1158,7 +1155,7 @@
     </row>
     <row r="34" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I34">
         <v>67</v>
@@ -1167,7 +1164,7 @@
         <v>79</v>
       </c>
       <c r="AG34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1175,7 +1172,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D35">
         <v>82</v>
@@ -1184,7 +1181,7 @@
         <v>104</v>
       </c>
       <c r="AL35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AM35">
         <v>2</v>
@@ -1192,7 +1189,7 @@
     </row>
     <row r="36" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F36">
         <v>73</v>
@@ -1201,7 +1198,7 @@
         <v>79</v>
       </c>
       <c r="AJ36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1209,7 +1206,7 @@
         <v>15</v>
       </c>
       <c r="C37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D37">
         <v>71</v>
@@ -1218,7 +1215,7 @@
         <v>71</v>
       </c>
       <c r="AL37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AM37">
         <v>15</v>
@@ -1226,10 +1223,16 @@
     </row>
     <row r="39" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="O39" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="P39">
+        <v>63</v>
+      </c>
+      <c r="V39">
+        <v>69</v>
       </c>
       <c r="W39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1237,7 +1240,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D42">
         <v>114</v>
@@ -1246,7 +1249,7 @@
         <v>101</v>
       </c>
       <c r="AL42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AM42">
         <v>1</v>
@@ -1254,7 +1257,7 @@
     </row>
     <row r="43" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F43">
         <v>72</v>
@@ -1263,7 +1266,7 @@
         <v>95</v>
       </c>
       <c r="AJ43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1271,19 +1274,19 @@
         <v>16</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D44">
         <v>55</v>
       </c>
       <c r="R44" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="AK44">
         <v>80</v>
       </c>
       <c r="AL44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AM44">
         <v>16</v>
@@ -1291,7 +1294,7 @@
     </row>
     <row r="45" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I45">
         <v>77</v>
@@ -1300,7 +1303,7 @@
         <v>90</v>
       </c>
       <c r="AG45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1308,19 +1311,19 @@
         <v>8</v>
       </c>
       <c r="C46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D46">
         <v>61</v>
       </c>
       <c r="R46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AK46">
         <v>77</v>
       </c>
       <c r="AL46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AM46">
         <v>8</v>
@@ -1328,7 +1331,7 @@
     </row>
     <row r="47" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F47">
         <v>73</v>
@@ -1337,7 +1340,7 @@
         <v>72</v>
       </c>
       <c r="AJ47" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1345,7 +1348,7 @@
         <v>9</v>
       </c>
       <c r="C48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D48">
         <v>67</v>
@@ -1354,7 +1357,7 @@
         <v>102</v>
       </c>
       <c r="AL48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AM48">
         <v>9</v>
@@ -1362,7 +1365,7 @@
     </row>
     <row r="49" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L49">
         <v>59</v>
@@ -1371,7 +1374,7 @@
         <v>95</v>
       </c>
       <c r="AD49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1379,19 +1382,19 @@
         <v>5</v>
       </c>
       <c r="C50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D50">
         <v>78</v>
       </c>
       <c r="S50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AK50">
         <v>91</v>
       </c>
       <c r="AL50" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AM50">
         <v>5</v>
@@ -1399,7 +1402,7 @@
     </row>
     <row r="51" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F51">
         <v>72</v>
@@ -1408,7 +1411,7 @@
         <v>65</v>
       </c>
       <c r="AJ51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1416,7 +1419,7 @@
         <v>12</v>
       </c>
       <c r="C52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D52">
         <v>68</v>
@@ -1425,7 +1428,7 @@
         <v>71</v>
       </c>
       <c r="AL52" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AM52">
         <v>12</v>
@@ -1433,7 +1436,7 @@
     </row>
     <row r="53" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H53" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I53">
         <v>71</v>
@@ -1442,7 +1445,7 @@
         <v>77</v>
       </c>
       <c r="AG53" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="54" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1450,19 +1453,19 @@
         <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D54">
         <v>76</v>
       </c>
       <c r="R54" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AK54">
         <v>90</v>
       </c>
       <c r="AL54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AM54">
         <v>4</v>
@@ -1470,7 +1473,7 @@
     </row>
     <row r="55" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F55">
         <v>74</v>
@@ -1479,7 +1482,7 @@
         <v>90</v>
       </c>
       <c r="AJ55" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1487,7 +1490,7 @@
         <v>13</v>
       </c>
       <c r="C56" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D56">
         <v>47</v>
@@ -1496,7 +1499,7 @@
         <v>70</v>
       </c>
       <c r="AL56" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AM56">
         <v>13</v>
@@ -1504,10 +1507,10 @@
     </row>
     <row r="57" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O57">
         <v>62</v>
@@ -1516,10 +1519,10 @@
         <v>91</v>
       </c>
       <c r="AA57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AD57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1527,7 +1530,7 @@
         <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D58">
         <v>78</v>
@@ -1536,7 +1539,7 @@
         <v>78</v>
       </c>
       <c r="AL58" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AM58">
         <v>6</v>
@@ -1544,7 +1547,7 @@
     </row>
     <row r="59" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E59" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F59">
         <v>55</v>
@@ -1553,7 +1556,7 @@
         <v>79</v>
       </c>
       <c r="AJ59" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="60" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1561,7 +1564,7 @@
         <v>11</v>
       </c>
       <c r="C60" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D60">
         <v>82</v>
@@ -1570,7 +1573,7 @@
         <v>56</v>
       </c>
       <c r="AL60" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AM60">
         <v>11</v>
@@ -1578,7 +1581,7 @@
     </row>
     <row r="61" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I61">
         <v>65</v>
@@ -1587,7 +1590,7 @@
         <v>76</v>
       </c>
       <c r="AG61" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="62" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1595,7 +1598,7 @@
         <v>3</v>
       </c>
       <c r="C62" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D62">
         <v>105</v>
@@ -1604,7 +1607,7 @@
         <v>82</v>
       </c>
       <c r="AL62" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AM62">
         <v>3</v>
@@ -1612,7 +1615,7 @@
     </row>
     <row r="63" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E63" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F63">
         <v>76</v>
@@ -1621,7 +1624,7 @@
         <v>72</v>
       </c>
       <c r="AJ63" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1629,7 +1632,7 @@
         <v>14</v>
       </c>
       <c r="C64" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D64">
         <v>70</v>
@@ -1638,7 +1641,7 @@
         <v>73</v>
       </c>
       <c r="AL64" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AM64">
         <v>14</v>
@@ -1646,7 +1649,7 @@
     </row>
     <row r="65" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K65" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L65">
         <v>71</v>
@@ -1655,7 +1658,7 @@
         <v>62</v>
       </c>
       <c r="AD65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="66" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1663,7 +1666,7 @@
         <v>7</v>
       </c>
       <c r="C66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D66">
         <v>50</v>
@@ -1672,7 +1675,7 @@
         <v>89</v>
       </c>
       <c r="AL66" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AM66">
         <v>7</v>
@@ -1680,7 +1683,7 @@
     </row>
     <row r="67" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F67">
         <v>57</v>
@@ -1689,7 +1692,7 @@
         <v>63</v>
       </c>
       <c r="AJ67" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="68" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1697,7 +1700,7 @@
         <v>10</v>
       </c>
       <c r="C68" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D68">
         <v>63</v>
@@ -1706,7 +1709,7 @@
         <v>84</v>
       </c>
       <c r="AL68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AM68">
         <v>10</v>
@@ -1714,7 +1717,7 @@
     </row>
     <row r="69" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I69">
         <v>55</v>
@@ -1723,7 +1726,7 @@
         <v>62</v>
       </c>
       <c r="AG69" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="70" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1731,7 +1734,7 @@
         <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D70">
         <v>78</v>
@@ -1740,7 +1743,7 @@
         <v>108</v>
       </c>
       <c r="AL70" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AM70">
         <v>2</v>
@@ -1748,7 +1751,7 @@
     </row>
     <row r="71" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E71" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F71">
         <v>88</v>
@@ -1757,7 +1760,7 @@
         <v>82</v>
       </c>
       <c r="AJ71" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="72" spans="2:39" x14ac:dyDescent="0.55000000000000004">
@@ -1765,7 +1768,7 @@
         <v>15</v>
       </c>
       <c r="C72" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D72">
         <v>47</v>
@@ -1774,7 +1777,7 @@
         <v>74</v>
       </c>
       <c r="AL72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM72">
         <v>15</v>

</xml_diff>